<commit_message>
Paper Summary sheet Updated
</commit_message>
<xml_diff>
--- a/BdsL_paper_Summary.xlsx
+++ b/BdsL_paper_Summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BDSL_CapstonProject_\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4957EEEB-AA9B-4D74-A382-FF66A99338E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3B4A360-2FE8-44D4-9A6D-8B310E5DB656}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{B9C80F48-A763-4B93-A58D-04AE71AFC590}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B9C80F48-A763-4B93-A58D-04AE71AFC590}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
   <si>
     <t>Paper Title</t>
   </si>
@@ -54,13 +54,154 @@
   </si>
   <si>
     <t>Result</t>
+  </si>
+  <si>
+    <t>BAUST Lipi: A BdSL Dataset with Deep Learning Based Bangla Sign Language Recognition</t>
+  </si>
+  <si>
+    <t>Created a new, comprehensive BdSL dataset (BAUST Lipi) and devised a hybrid CNN-LSTM model to solve the problem of achieving high-performance accuracy in BdSL recognition</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> BDSL 49: A comprehensive dataset of Bangla sign language</t>
+  </si>
+  <si>
+    <t>BDSL 49, consisting of 29,490 images across 49 classes of Bengali alphabets, numeric characters, and special characters</t>
+  </si>
+  <si>
+    <t>Provided a freely available, comprehensive 49-class dataset to enable researchers to train and evaluate machine learning models specifically for Bengali Sign Language</t>
+  </si>
+  <si>
+    <t>The YOLOv4 model achieved 99.4% accuracy (99.9% mean average precision) for detection, and the Xception model achieved the highest recognition accuracy at 93%</t>
+  </si>
+  <si>
+    <t>BdSLW60: A Word-Level Bangla Sign Language Dataset</t>
+  </si>
+  <si>
+    <t>BdSLW60, a word-level dataset containing 9,307 video trials of 60 Bengali sign words performed by 18 signers in an unconstrained setting</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Extracted landmark-based features (pose, face, and hands) using Google MediaPipe, and applied a unique relative quantization-based key frame encoding technique. Evaluated using SVM, SVM-DTW, and an attention-based bi-LSTM network</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Addressed the scarcity of word-level BdSL datasets by creating BdSLW60 and proposed a novel relative quantization approach for continuous sign language recognition</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Benchmarking showed a testing accuracy of up to 67.6% using SVM and up to 75.1% using the attention-based bi-LSTM</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Bilingual Sign Language Recognition: A YOLOv11-Based Model for Bangla and English Alphabets</t>
+  </si>
+  <si>
+    <t>A custom open-source dataset of 9,556 images representing 64 distinct letter signs from both Bangla Sign Language (BdSL) and American Sign Language (ASL)</t>
+  </si>
+  <si>
+    <t>Utilized the state-of-the-art YOLOv11 object detection architecture for real-time recognition. Data augmentation (cropping, rotation, brightness correction) was applied to enhance generalizability</t>
+  </si>
+  <si>
+    <t>Introduced a unified bilingual detection system capable of recognizing both BdSL and ASL alphabets concurrently in real-time to enhance interlingual communication</t>
+  </si>
+  <si>
+    <t>Dynamic BDSL Digit Recognition Using Hybrid 3DCNN+BiLSTM Model</t>
+  </si>
+  <si>
+    <t>Not explicitly stated (recent based on context).</t>
+  </si>
+  <si>
+    <t>A subset of the SignBD-Word dataset utilizing 11 numeral Bengali digit signs composed of extracted RGB human body pose keypoints skeleton data</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> A hybrid architecture combining 3DCNN and bidirectional LSTM (BiLSTM) layers, utilizing DenseNet-201 as a base feature extractor for classifying body joint skeleton motion patterns</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> The ensemble model (DenseNet-201+3DCNN+BiLSTM) achieved the highest scores (Precision 0.37, Recall 0.36, F1-Score 0.33), which increased accuracy by 4.54% compared to using DenseNet-201+BiLSTM alone</t>
+  </si>
+  <si>
+    <t>Pioneered the implementation of DenseNet-201 combined with 3DCNN and BiLSTM for dynamic BdSL digit recognition based on skeleton motion patterns</t>
+  </si>
+  <si>
+    <t>IsharaNet: A robust nested feature fusion coupled with attention incorporated width scaled lightweight architecture for Bengali sign language recognition</t>
+  </si>
+  <si>
+    <t>Evaluated across four datasets: BdSL47, BdSLW-11, Shongket, and KU-BdSL</t>
+  </si>
+  <si>
+    <t>Proposed IsharaNet, a lightweight deep neural network architecture leveraging parallel convolutional operations, nested feature fusion, and spatial/channel attention mechanisms</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Introduced a highly efficient, width-scaled lightweight architecture capable of accurately capturing complex gesture semantics across Bengali sign alphabets, numerals, and words</t>
+  </si>
+  <si>
+    <t>Achieved top accuracies of 99.85% for numerals, 99.77% for alphabets, and 99.09% for words, with a consistent AUC score of 0.999 across tasks, outperforming state-of-the-art models</t>
+  </si>
+  <si>
+    <t>KU-BdSL: An open dataset for Bengali sign language recognition</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> KU-BdSL, consisting of 1,500 images categorized into 30 classes representing 38 Bengali consonants captured by 39 participants</t>
+  </si>
+  <si>
+    <t>Dataset creation and formatting. Images were captured using smartphone cameras under various lighting conditions and backgrounds. The dataset was structured into Uni-scale (USLD), Multi-scale (MSLD), and Annotated (AMSLD) formats utilizing DarkNet annotations</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Provided a reliable, well-structured, and open dataset focused on static single-hand gestures of Bengali consonants to facilitate the development of machine translation solutions</t>
+  </si>
+  <si>
+    <t>Successfully published the annotated dataset for public research use, paving the way for image or video-based consonant identification</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Recognition of Bangladeshi Sign Language (BdSL) Words using Deep Convolutional Neural Networks (DCNNs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> A custom dataset of 992 images representing 10 frequently used BdSL words created by the authors</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Image preprocessing (rescaling, flipping, shearing) combined with training deep learning/transfer learning models including a modified CNN, DenseNet201, ResNet50-V2, and MobileNet-V2</t>
+  </si>
+  <si>
+    <t>Focused specifically on real-time BdSL word detection (rather than just characters or digits) to bridge the communication gap for the deaf and dumb community</t>
+  </si>
+  <si>
+    <t>DenseNet201 and ResNet50-V2 both achieved testing accuracies of 93%, outperforming the custom CNN (76%) and MobileNet-V2 (87%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Transformer based sign-to-text translation for Bangladeshi sign language</t>
+  </si>
+  <si>
+    <t>A custom dataset of 102 common BdSL words, converted into 91,800 landmark sequences (30 frames per video)</t>
+  </si>
+  <si>
+    <t>A feature-first pipeline using Google MediaPipe to extract 258 skeletal landmarks (hands and upper body) per frame. These sequences were classified using a lightweight Transformer encoder leveraging positional information and self-attention</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Standardized a reproducible, privacy-friendly data curation pipeline and introduced a compact, real-time Transformer model capable of modeling temporal structure directly over skeletal landmarks for 102 BdSL words</t>
+  </si>
+  <si>
+    <t>The Transformer model achieved 98.12% test accuracy, significantly outperforming baselines such as Sequential LSTM (81.21%) and SSD MobileNet V2 (78.02%)</t>
+  </si>
+  <si>
+    <t>BAUST Lipi, comprising 18,000 images covering 36 Bengali symbols (30 consonants and 6 vowels)</t>
+  </si>
+  <si>
+    <t>A hybrid Convolutional Neural Network (CNN) model integrated with multiple convolutional layers, dropout techniques, and LSTM layers</t>
+  </si>
+  <si>
+    <t>The proposed hybrid CNN-LSTM model achieved a testing accuracy rate of 97.28% (97.92% overall accuracy)</t>
+  </si>
+  <si>
+    <t>The study utilized YOLOv4 for real-time hand sign detection from full-frame images and tested multiple pre-trained deep learning models (Xception, InceptionV3, InceptionResNetv2, ResNet50V2, DenseNet) for cropped image recognition</t>
+  </si>
+  <si>
+    <t>The YOLOv11 model outperformed previous YOLO versions (v8, v9, v10, v12), achieving a precision of 99.12%, recall of 99.63%, and mAP of 99.4%</t>
+  </si>
+  <si>
+    <t>s</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -69,19 +210,54 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="20"/>
+      <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF303030"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color rgb="FF303030"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -96,13 +272,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -438,36 +626,235 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91718BDA-A7AF-4253-B864-230AF643558B}">
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:I18"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="27.6328125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="18.54296875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="12.54296875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="44.81640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="48.08984375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="41.26953125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="34.7265625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="28.90625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="9.54296875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="48.54296875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="53.54296875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="45" style="1" customWidth="1"/>
     <col min="7" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="2" customFormat="1" ht="26" x14ac:dyDescent="0.6">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:6" ht="20.5" x14ac:dyDescent="0.45">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="6" t="s">
         <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="66" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" s="3">
+        <v>2024</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="99" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="99" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="115.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="2">
+        <v>2025</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" s="5"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+    </row>
+    <row r="13" spans="1:6" ht="93" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" s="5"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+    </row>
+    <row r="15" spans="1:6" ht="93" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="93" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C16" s="1">
+        <v>2023</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="62" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17" s="1">
+        <v>2023</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="77.5" x14ac:dyDescent="0.35">
+      <c r="A18" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>